<commit_message>
결과 파일 업데이트 2026-09-04 06:36
</commit_message>
<xml_diff>
--- a/results/andar_할인율모니터링_20260904.xlsx
+++ b/results/andar_할인율모니터링_20260904.xlsx
@@ -571,7 +571,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>3,526</t>
+          <t>3,529</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -613,7 +613,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>3,526</t>
+          <t>3,529</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1247,84 +1247,84 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16649&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9023&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>EPTBG-02</t>
+          <t>EMTBG-03</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>서밋 유틸리티 백팩</t>
+          <t>숄더 앤 크로스백</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>89,000</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>62,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>51%</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>107</t>
+          <t>8,009</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9023&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16649&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>EMTBG-03</t>
+          <t>EPTBG-02</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>숄더 앤 크로스백</t>
+          <t>서밋 유틸리티 백팩</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>89,000</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>62,000</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>51%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>8,009</t>
+          <t>107</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>410</t>
+          <t>411</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2,369</t>
+          <t>2,371</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1499,84 +1499,84 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10940&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15403&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ENTBG-03</t>
+          <t>EOTBG-21</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>데일리 스트링 쇼퍼백</t>
+          <t>데일리 라운드백</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>75,000</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>49,500</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>34%</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>721</t>
+          <t>110</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15403&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10940&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>EOTBG-21</t>
+          <t>ENTBG-03</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>데일리 라운드백</t>
+          <t>데일리 스트링 쇼퍼백</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>75,000</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>49,500</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>34%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>110</t>
+          <t>722</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
@@ -1613,7 +1613,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>6,570</t>
+          <t>6,571</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1781,7 +1781,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>425</t>
+          <t>426</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2171,126 +2171,126 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17437&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8838&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>EPTCP-03</t>
+          <t>EMTSV-03</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>썬가드 와이드 버킷햇</t>
+          <t>[1&amp;1] 서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>27,800</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>22,900</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>1,997</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8838&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15143&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>EMTSV-03</t>
+          <t>EOTBG-17</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>[1&amp;1] 서포트 무릎 보호대</t>
+          <t>3 in 1 캐리온 더플백</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>27,800</t>
+          <t>109,000</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>22,900</t>
+          <t>76,500</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>30%</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>1,995</t>
+          <t>41</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17425&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15371&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>EPTSC-06</t>
+          <t>EOTBG-15</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>필라테스 크루 삭스</t>
+          <t>폴더블 짐백 2.0</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>40,500</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>31%</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>74</t>
+          <t>54</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -2327,7 +2327,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>3,017</t>
+          <t>3,019</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>3,017</t>
+          <t>3,019</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2381,27 +2381,27 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15629&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16844&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>EOTBG-23</t>
+          <t>EPTET-02</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>안다르 실버 리유저블백 M</t>
+          <t>언더웨어 세탁망</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>6,500</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>6,500</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>364</t>
+          <t>285</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -2423,69 +2423,69 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15143&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15409&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>EOTBG-17</t>
+          <t>EOTSC-15</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>3 in 1 캐리온 더플백</t>
+          <t>논슬립 퍼포먼스 풀 토삭스</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>109,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>76,500</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>41</t>
+          <t>151</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15409&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17425&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>EOTSC-15</t>
+          <t>EPTSC-06</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 풀 토삭스</t>
+          <t>필라테스 크루 삭스</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -2495,81 +2495,81 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>74</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15371&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17437&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>EOTBG-15</t>
+          <t>EPTCP-03</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>폴더블 짐백 2.0</t>
+          <t>썬가드 와이드 버킷햇</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>40,500</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>59</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16844&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15629&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>EPTET-02</t>
+          <t>EOTBG-23</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>언더웨어 세탁망</t>
+          <t>안다르 실버 리유저블백 M</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>6,500</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>6,500</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>285</t>
+          <t>364</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -2633,153 +2633,153 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15350&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15370&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>EOTSC-09</t>
+          <t>EOTBG-14</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>[1&amp;1] 컴프레션 러닝 니삭스</t>
+          <t>폴더블 캐리백 2.0</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>24,900</t>
+          <t>49,500</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>28%</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>670</t>
+          <t>86</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13215&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15350&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>EOTCP-01</t>
+          <t>EOTSC-09</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>올라운드 버킷햇</t>
+          <t>[1&amp;1] 컴프레션 러닝 니삭스</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>24,900</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>353</t>
+          <t>670</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15370&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6660&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>EOTBG-14</t>
+          <t>EKPMT-03</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>폴더블 캐리백 2.0</t>
+          <t>릴렉스 논슬립 요가 타월</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>35,900</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>49,500</t>
+          <t>35,900</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>86</t>
+          <t>1,551</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6660&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13215&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>EKPMT-03</t>
+          <t>EOTCP-01</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>릴렉스 논슬립 요가 타월</t>
+          <t>올라운드 버킷햇</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>35,900</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>35,900</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2789,12 +2789,12 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>1,551</t>
+          <t>353</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
@@ -2843,27 +2843,27 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17423&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15408&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>EPTSC-04</t>
+          <t>EOTSC-14</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>필라테스 토삭스</t>
+          <t>맨즈 논슬립 풀 토삭스</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
@@ -2873,39 +2873,39 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>94</t>
+          <t>102</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15408&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17423&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>EOTSC-14</t>
+          <t>EPTSC-04</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>맨즈 논슬립 풀 토삭스</t>
+          <t>필라테스 토삭스</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2915,12 +2915,12 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>102</t>
+          <t>94</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -2969,121 +2969,121 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9989&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>EMTET-02</t>
+          <t>EOTSC-16</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>소프트 쿠셔닝 훌라후프</t>
+          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>25,800</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>23%</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>621</t>
+          <t>511</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13854&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>EOTSC-06</t>
+          <t>EOTSC-17</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>서포트 쿠션 러닝 삭스</t>
+          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>25,800</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>23%</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>758</t>
+          <t>511</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13604&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9989&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>EOTSV-01</t>
+          <t>EMTET-02</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>[1&amp;1] 하이 서포트 무릎 보호대</t>
+          <t>소프트 쿠셔닝 훌라후프</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>24,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>701</t>
+          <t>621</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
@@ -3095,79 +3095,79 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13854&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>EOTSC-16</t>
+          <t>EOTSC-06</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
+          <t>서포트 쿠션 러닝 삭스</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>25,800</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>23%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>511</t>
+          <t>758</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15385&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=5144&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>EOTSC-17</t>
+          <t>EJPMS-05</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>[1&amp;1] 논슬립 스킨 토삭스</t>
+          <t>릴렉스 마사지 스틱 Ⅱ</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>25,800</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>23%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>511</t>
+          <t>10,356</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
@@ -3251,7 +3251,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>244</t>
+          <t>245</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
@@ -3263,37 +3263,37 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13852&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13604&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>EOTET-03</t>
+          <t>EOTSV-01</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>라이트 러닝 베스트</t>
+          <t>[1&amp;1] 하이 서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>24,900</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>701</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -3305,27 +3305,27 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16631&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>EPTSV-03</t>
+          <t>EMTRB-01</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>컴프레션 카프 슬리브 (종아리 보호대)</t>
+          <t>서포트 힙 밴드</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>238</t>
+          <t>1,364</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>EMTRB-01</t>
+          <t>EMTRB-02</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3394,7 +3394,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>EMTRB-02</t>
+          <t>EMTRB-03</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3431,27 +3431,27 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10188&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13852&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EMTRB-03</t>
+          <t>EOTET-03</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>서포트 힙 밴드</t>
+          <t>라이트 러닝 베스트</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -3461,39 +3461,39 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>1,364</t>
+          <t>98</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=5144&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16631&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>EJPMS-05</t>
+          <t>EPTSV-03</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>릴렉스 마사지 스틱 Ⅱ</t>
+          <t>컴프레션 카프 슬리브 (종아리 보호대)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>10,356</t>
+          <t>238</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -3515,27 +3515,27 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14561&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8621&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EOTBG-05</t>
+          <t>EMTSV-06</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>메쉬 포켓 비치백</t>
+          <t>에어쿨링 손목 보호대</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>49,000</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -3545,39 +3545,39 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>1,081</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8621&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14561&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>EMTSV-06</t>
+          <t>EOTBG-05</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>에어쿨링 손목 보호대</t>
+          <t>메쉬 포켓 비치백</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>49,000</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -3587,207 +3587,207 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>1,081</t>
+          <t>56</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15153&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>EOTSC-13</t>
+          <t>ENTSC-19</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>테이핑 테크 러닝 삭스</t>
+          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>16,900</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>272</t>
+          <t>304</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10948&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>ENTSC-20</t>
+          <t>EOTSC-14</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>시그니처 로고 크루 삭스</t>
+          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>16,900</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>565</t>
+          <t>304</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15377&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ENTSC-19</t>
+          <t>EOTGL-04</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
+          <t>논슬립 스킨 요기 글러브</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>16,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>304</t>
+          <t>188</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15431&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10948&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>EOTSC-14</t>
+          <t>ENTSC-20</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>[1&amp;1] 맨즈 논슬립 토삭스</t>
+          <t>시그니처 로고 크루 삭스</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>16,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>304</t>
+          <t>565</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15377&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15153&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>EOTGL-04</t>
+          <t>EOTSC-13</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>논슬립 스킨 요기 글러브</t>
+          <t>테이핑 테크 러닝 삭스</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -3797,39 +3797,39 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>188</t>
+          <t>272</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6661&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13410&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>EKPMB-01</t>
+          <t>EOTSC-09</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>릴렉스 웨이트볼 0.5kg</t>
+          <t>컴프레션 러닝 니삭스</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3839,39 +3839,39 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>689</t>
+          <t>345</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13410&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12765&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>EOTSC-09</t>
+          <t>ENTBG-16</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>컴프레션 러닝 니삭스</t>
+          <t>라이트 패딩 쇼퍼백</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>69,000</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -3881,39 +3881,39 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>345</t>
+          <t>623</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12765&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6661&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>ENTBG-16</t>
+          <t>EKPMB-01</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>라이트 패딩 쇼퍼백</t>
+          <t>릴렉스 웨이트볼 0.5kg</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>69,000</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3923,123 +3923,123 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>623</t>
+          <t>689</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6664&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8799&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>EKPRB-04</t>
+          <t>EMTFB-01</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>릴렉스 3레벨 스트레칭 롱밴드</t>
+          <t>[3 SET] 에어쿨링 스크런치</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>34,900</t>
+          <t>17,700</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>34,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>21%</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>467</t>
+          <t>1,639</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11458&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8799&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>ENTSC-13</t>
+          <t>ENTFB-02</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 크루삭스</t>
+          <t>[3 SET] 에어쿨링 스크런치</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>17,700</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>21%</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>662</t>
+          <t>1,639</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8578&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16650&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>EMTSC-01</t>
+          <t>EPTCP-02</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>링글 크루 삭스</t>
+          <t>시그니처 로고 나일론 볼캡</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -4049,39 +4049,39 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>1,323</t>
+          <t>58</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16637&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6664&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EPTFB-02</t>
+          <t>EKPRB-04</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>퍼포먼스 심리스 손목밴드</t>
+          <t>릴렉스 3레벨 스트레칭 롱밴드</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>34,900</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>34,900</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4091,39 +4091,39 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>264</t>
+          <t>467</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16650&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16637&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>EPTCP-02</t>
+          <t>EPTFB-02</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>시그니처 로고 나일론 볼캡</t>
+          <t>퍼포먼스 심리스 손목밴드</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4133,81 +4133,81 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>264</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6828&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6662&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>EKPET-01</t>
+          <t>EKPMB-02</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>[1&amp;1] 릴렉스 소프트 웨이트바 1kg</t>
+          <t>릴렉스 미니 짐볼</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>41,800</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>35,600</t>
+          <t>13,000</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>593</t>
+          <t>1,224</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16847&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11458&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EPTSC-02</t>
+          <t>ENTSC-13</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>하이 쿠션 테이핑 러닝 삭스</t>
+          <t>논슬립 퍼포먼스 크루삭스</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -4217,7 +4217,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>89</t>
+          <t>664</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
@@ -4229,27 +4229,27 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6662&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16847&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>EKPMB-02</t>
+          <t>EPTSC-02</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>릴렉스 미니 짐볼</t>
+          <t>하이 쿠션 테이핑 러닝 삭스</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>13,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -4259,39 +4259,39 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>1,224</t>
+          <t>89</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13404&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11039&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EOTGL-01</t>
+          <t>ENTFB-01</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>짐 글러브 2.0</t>
+          <t>에어쿨링 라인 스크런치</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>25,000</t>
+          <t>8,900</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -4301,7 +4301,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>285</t>
+          <t>758</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
@@ -4313,27 +4313,27 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11039&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8578&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>ENTFB-01</t>
+          <t>EMTSC-01</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>에어쿨링 라인 스크런치</t>
+          <t>링글 크루 삭스</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>8,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
@@ -4343,7 +4343,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>754</t>
+          <t>1,323</t>
         </is>
       </c>
       <c r="H94" t="inlineStr">
@@ -4355,37 +4355,37 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8727&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6828&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>EMTSC-04</t>
+          <t>EKPET-01</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>논슬립 서포트 하프 토삭스 (HOLE)</t>
+          <t>[1&amp;1] 릴렉스 소프트 웨이트바 1kg</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>41,800</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>10,900</t>
+          <t>35,600</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>15%</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>643</t>
+          <t>594</t>
         </is>
       </c>
       <c r="H95" t="inlineStr">
@@ -4397,37 +4397,37 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11457&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11130&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>ENTSC-12</t>
+          <t>ENTSV-01</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 토삭스</t>
+          <t>[1&amp;1] 3D 쿨링 팔토시</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>25,900</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>13%</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>4,135</t>
+          <t>547</t>
         </is>
       </c>
       <c r="H96" t="inlineStr">
@@ -4439,37 +4439,37 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8837&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11457&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>EMTSV-02</t>
+          <t>ENTSC-12</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>[1&amp;1] 서포트 발목 보호대</t>
+          <t>논슬립 퍼포먼스 토삭스</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>27,800</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>22,900</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>710</t>
+          <t>4,135</t>
         </is>
       </c>
       <c r="H97" t="inlineStr">
@@ -4481,37 +4481,37 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8799&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8727&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>EMTFB-01</t>
+          <t>EMTSC-04</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>[3 SET] 에어쿨링 스크런치</t>
+          <t>논슬립 서포트 하프 토삭스 (HOLE)</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>17,700</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>10,900</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>21%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>1,639</t>
+          <t>643</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
@@ -4523,111 +4523,111 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8799&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13407&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ENTFB-02</t>
+          <t>EOTSV-03</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>[3 SET] 에어쿨링 스크런치</t>
+          <t>서포트 허리 보호대</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>17,700</t>
+          <t>34,000</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>34,000</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>21%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>1,639</t>
+          <t>173</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11130&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13404&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ENTSV-01</t>
+          <t>EOTGL-01</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>[1&amp;1] 3D 쿨링 팔토시</t>
+          <t>짐 글러브 2.0</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>25,900</t>
+          <t>25,000</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>547</t>
+          <t>285</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13407&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13842&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>EOTSV-03</t>
+          <t>EOTBG-04</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>서포트 허리 보호대</t>
+          <t>데님 포켓 숄더백</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>34,000</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>34,000</t>
+          <t>59,000</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -4637,39 +4637,39 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>39</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13851&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13859&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>EOTCP-03</t>
+          <t>ENTSO-12</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>쿨 라운드 볼캡</t>
+          <t>안다르 제트플라이 (맨즈)</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>139,000</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>45,000</t>
+          <t>139,000</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -4679,39 +4679,39 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>98</t>
+          <t>694</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13405&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13851&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>EOTSV-01</t>
+          <t>EOTCP-03</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>하이 서포트 무릎 보호대</t>
+          <t>쿨 라운드 볼캡</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>45,000</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -4721,39 +4721,39 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>701</t>
+          <t>98</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17440&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8728&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>EPTET-03</t>
+          <t>EMTSC-05</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>안다르 3단 양우산</t>
+          <t>논슬립 서포트 하프 토삭스 (SOLID)</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>9,900</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -4763,81 +4763,81 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>559</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>4.4</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17424&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8837&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>EPTSC-05</t>
+          <t>EMTSV-02</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>필라테스 앵클 삭스</t>
+          <t>[1&amp;1] 서포트 발목 보호대</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>27,800</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>22,900</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>710</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8728&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13405&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>EMTSC-05</t>
+          <t>EOTSV-01</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>논슬립 서포트 하프 토삭스 (SOLID)</t>
+          <t>하이 서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>9,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -4847,39 +4847,39 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>559</t>
+          <t>701</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13842&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17424&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>EOTBG-04</t>
+          <t>EPTSC-05</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>데님 포켓 숄더백</t>
+          <t>필라테스 앵클 삭스</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>59,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -4901,22 +4901,22 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10953&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17440&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>ENTSC-07</t>
+          <t>EPTET-03</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>[3 SET] 에어컴피 크루 삭스</t>
+          <t>안다르 3단 양우산</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>51,000</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -4926,44 +4926,44 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>558</t>
+          <t>35</t>
         </is>
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.4</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15375&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=16660&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>EOTSC-16</t>
+          <t>EOTET-03</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>논슬립 스킨 하프 토삭스</t>
+          <t>맨즈 라이트 러닝 베스트</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>79,000</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
@@ -4973,39 +4973,39 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>107</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>4.9</t>
+          <t>4.6</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13859&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11459&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>ENTSO-12</t>
+          <t>ENTSC-14</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>안다르 제트플라이 (맨즈)</t>
+          <t>논슬립 퍼포먼스 니삭스</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>139,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>139,000</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F110" t="inlineStr">
@@ -5015,81 +5015,81 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>694</t>
+          <t>752</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15376&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10953&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>EOTSC-17</t>
+          <t>ENTSC-07</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>논슬립 스킨 토삭스</t>
+          <t>[3 SET] 에어컴피 크루 삭스</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>51,000</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>12,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>43%</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>85</t>
+          <t>558</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=16660&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15376&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>EOTET-03</t>
+          <t>EOTSC-17</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>맨즈 라이트 러닝 베스트</t>
+          <t>논슬립 스킨 토삭스</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>79,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F112" t="inlineStr">
@@ -5099,39 +5099,39 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>85</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>4.6</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11459&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12778&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>ENTSC-14</t>
+          <t>ENTBG-14</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>논슬립 퍼포먼스 니삭스</t>
+          <t>웨이브 패딩 파우치</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="F113" t="inlineStr">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>752</t>
+          <t>191</t>
         </is>
       </c>
       <c r="H113" t="inlineStr">
@@ -5225,7 +5225,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>5,106</t>
+          <t>5,108</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -5321,27 +5321,27 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=10554&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15375&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>ENTMK-01</t>
+          <t>EOTSC-16</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>UV 프로텍션 맨즈 골프 마스크</t>
+          <t>논슬립 스킨 하프 토삭스</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>23,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>23,000</t>
+          <t>12,900</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -5351,39 +5351,39 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>1,534</t>
+          <t>107</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.9</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14085&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=10554&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>EOTSV-04</t>
+          <t>ENTMK-01</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>프리런 라이트 러닝 밴드</t>
+          <t>UV 프로텍션 맨즈 골프 마스크</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>23,000</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>23,000</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -5393,12 +5393,12 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>1,534</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -5447,79 +5447,79 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13605&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14085&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>EOTSV-02</t>
+          <t>EOTSV-04</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>[1&amp;1] 하이 서포트 팔꿈치 보호대</t>
+          <t>프리런 라이트 러닝 밴드</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>29,800</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>24,900</t>
+          <t>32,000</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>16%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>125</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.2</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6665&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13605&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>EKPRB-05</t>
+          <t>EOTSV-02</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>릴렉스 4레벨 힙 밴드</t>
+          <t>[1&amp;1] 하이 서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>21,900</t>
+          <t>29,800</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>21,900</t>
+          <t>24,900</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>16%</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>527</t>
+          <t>154</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -5531,27 +5531,27 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13566&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8769&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>EOTSC-10</t>
+          <t>EMTSV-02</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>시그니처 로고 맨즈 크루 삭스</t>
+          <t>서포트 발목 보호대</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>7,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -5561,91 +5561,91 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>710</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8836&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13566&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>EMTSV-01</t>
+          <t>EOTSC-10</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>[1&amp;1] 서포트 팔꿈치 보호대</t>
+          <t>시그니처 로고 맨즈 크루 삭스</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>27,800</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>22,900</t>
+          <t>7,900</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>18%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>588</t>
+          <t>213</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8769&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8836&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>EMTSV-02</t>
+          <t>EMTSV-01</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>서포트 발목 보호대</t>
+          <t>[1&amp;1] 서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>27,800</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>22,900</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>18%</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>710</t>
+          <t>588</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -5783,69 +5783,69 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=9996&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17857&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>EMTSC-27</t>
+          <t>EPTSC-03</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>올라운드 오버 니삭스</t>
+          <t>[1&amp;1] 데일리 루즈 삭스</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>23,800</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>18,900</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>21%</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>294</t>
+          <t>28</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13806&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8770&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>EOTSC-05</t>
+          <t>EMTSV-03</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>올데이 수피마 앵클 삭스</t>
+          <t>서포트 무릎 보호대</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>6,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -5855,81 +5855,81 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>471</t>
+          <t>1,997</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.5</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17857&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13806&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>EPTSC-03</t>
+          <t>EOTSC-05</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>[1&amp;1] 데일리 루즈 삭스</t>
+          <t>올데이 수피마 앵클 삭스</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>23,800</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>18,900</t>
+          <t>6,900</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>21%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>471</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8770&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=12096&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>EMTSV-03</t>
+          <t>ENTET-02</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>서포트 무릎 보호대</t>
+          <t>릴렉스 소프트 웨이트바 2kg</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>39,000</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -5939,39 +5939,39 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>1,995</t>
+          <t>76</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12096&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13406&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>ENTET-02</t>
+          <t>EOTSV-02</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>릴렉스 소프트 웨이트바 2kg</t>
+          <t>하이 서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>39,000</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -5981,39 +5981,39 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>154</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13805&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=9996&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>EOTSC-04</t>
+          <t>EMTSC-27</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>올데이 수피마 스니커즈 삭스</t>
+          <t>올라운드 오버 니삭스</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>5,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -6023,39 +6023,39 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>425</t>
+          <t>294</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13406&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6665&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>EOTSV-02</t>
+          <t>EKPRB-05</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>하이 서포트 팔꿈치 보호대</t>
+          <t>릴렉스 4레벨 힙 밴드</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>21,900</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -6065,7 +6065,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>154</t>
+          <t>527</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -6119,27 +6119,27 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11061&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13805&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>ENTSV-01</t>
+          <t>EOTSC-04</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>3D 쿨링 팔토시</t>
+          <t>올데이 수피마 스니커즈 삭스</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>5,900</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -6149,12 +6149,12 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>547</t>
+          <t>425</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -6203,27 +6203,27 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=11963&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11061&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>ENTSC-19</t>
+          <t>ENTSV-01</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>맨즈 논슬립 하프 토삭스</t>
+          <t>3D 쿨링 팔토시</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>11,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>92</t>
+          <t>547</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
@@ -6287,27 +6287,27 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=13408&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=11963&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>EOTSC-01</t>
+          <t>ENTSC-19</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>프레시 필드 니삭스</t>
+          <t>맨즈 논슬립 하프 토삭스</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>14,900</t>
+          <t>11,900</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -6317,39 +6317,39 @@
       </c>
       <c r="G141" t="inlineStr">
         <is>
-          <t>294</t>
+          <t>92</t>
         </is>
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17387&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=13408&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>EPTSC-08</t>
+          <t>EOTSC-01</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>맨즈 필라테스 크루 삭스</t>
+          <t>프레시 필드 니삭스</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>14,900</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
@@ -6359,29 +6359,29 @@
       </c>
       <c r="G142" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>294</t>
         </is>
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>5.0</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=17386&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17387&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>EPTSC-07</t>
+          <t>EPTSC-08</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>맨즈 필라테스 앵클 삭스</t>
+          <t>맨즈 필라테스 크루 삭스</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -6413,37 +6413,37 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=12778&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=15867&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>ENTBG-14</t>
+          <t>EOTSC-18</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>웨이브 패딩 파우치</t>
+          <t>[1&amp;1] 올데이 기모 삭스</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>21,800</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>32,000</t>
+          <t>15,900</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>27%</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>225</t>
         </is>
       </c>
       <c r="H144" t="inlineStr">
@@ -6455,69 +6455,69 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=15867&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14562&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>EOTSC-18</t>
+          <t>EOTBG-11</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>[1&amp;1] 올데이 기모 삭스</t>
+          <t>메쉬 파우치</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>21,800</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>15,900</t>
+          <t>29,000</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>190</t>
         </is>
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14562&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=6666&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>EOTBG-11</t>
+          <t>EKPET-01</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>메쉬 파우치</t>
+          <t>릴렉스 소프트 웨이트바 1kg</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>29,000</t>
+          <t>20,900</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -6527,39 +6527,39 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>594</t>
         </is>
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=6666&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=17386&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>EKPET-01</t>
+          <t>EPTSC-07</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>릴렉스 소프트 웨이트바 1kg</t>
+          <t>맨즈 필라테스 앵클 삭스</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>20,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
@@ -6569,39 +6569,39 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>593</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>5.0</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=14084&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=8768&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>EOTET-01</t>
+          <t>EMTSV-01</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>소프트 뱀부 롱 타월</t>
+          <t>서포트 팔꿈치 보호대</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>19,900</t>
+          <t>13,900</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -6611,39 +6611,39 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>588</t>
         </is>
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>4.8</t>
+          <t>4.7</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>https://andar.co.kr/product/detail.html?product_no=8768&amp;cate_no=2100&amp;display_group=1</t>
+          <t>https://andar.co.kr/product/detail.html?product_no=14084&amp;cate_no=2100&amp;display_group=1</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>EMTSV-01</t>
+          <t>EOTET-01</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>서포트 팔꿈치 보호대</t>
+          <t>소프트 뱀부 롱 타월</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>13,900</t>
+          <t>19,900</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -6653,12 +6653,12 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>588</t>
+          <t>236</t>
         </is>
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>4.7</t>
+          <t>4.8</t>
         </is>
       </c>
     </row>
@@ -6989,7 +6989,7 @@
       </c>
       <c r="G157" t="inlineStr">
         <is>
-          <t>6,361</t>
+          <t>6,362</t>
         </is>
       </c>
       <c r="H157" t="inlineStr">

</xml_diff>